<commit_message>
made some fixes with the logic
</commit_message>
<xml_diff>
--- a/Generated_Schedule.xlsx
+++ b/Generated_Schedule.xlsx
@@ -38,26 +38,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00BDD7EE"/>
         <bgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00CC99FF"/>
         <bgColor rgb="00CC99FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -544,22 +544,22 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>St.Paul's</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Vancouver General</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Brooke Richmond (4d)</t>
+          <t>Brooke Burnaby (2d)</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Surrey</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>WCMI Hornby (2d)</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Cranbrook (EKRH)</t>
+          <t>Medray (2d)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -587,22 +587,22 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Chilliwack</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>VMI Abbotsford/Langley (2d)</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>WCMI Kerrisdale (2d)</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>NSMI (4d)</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Richmond (4d)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>WCMI Hornby (2d)</t>
         </is>
@@ -632,22 +632,22 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>NSMI (4d)</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>VMI Abbotsford/Langley (2d)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Vancouver General</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Langley</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Greig Associates (2d)</t>
         </is>
@@ -679,22 +679,22 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
+          <t>Medray (2d)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Langley</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
           <t>Mission</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>WCMI Kerrisdale (2d)</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Greig Associates (2d)</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Langley</t>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Sechelt</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -724,22 +724,22 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Sechelt</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+          <t>Greig Associates (2d)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Delta</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
+          <t>Vancouver General</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
           <t>VMI Abbotsford/Langley (2d)</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Saanich</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -769,22 +769,22 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
+          <t>WCMI Hornby (2d)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Burnaby (2d)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
           <t>Saanich</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Mission</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>WCMI Hornby (2d)</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>WCMI Kerrisdale (2d)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -812,24 +812,24 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>Delta</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Medray (2d)</t>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Burnaby (2d)</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>St.Paul's</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Chilliwack</t>
+          <t>NSMI (4d)</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Eagle Ridge</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -857,24 +857,24 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Langley</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Greig Associates (2d)</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>WCMI Kerrisdale (2d)</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Medray (2d)</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>MSJ</t>
+          <t>Brooke Richmond (4d)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -904,22 +904,22 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Peace Arch</t>
+          <t>Brooke Richmond (4d)</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>WCMI Hornby (2d)</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
           <t>Vancouver General</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Chilliwack</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Lions Gate</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -947,24 +947,24 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Greig Associates (2d)</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Langley</t>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>NSMI (4d)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Mission</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Brooke Burnaby (2d)</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Squamish</t>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Campbell River</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -992,22 +992,22 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Brooke Richmond (4d)</t>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>WCMI Kerrisdale (2d)</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Delta</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
+          <t>Greig Associates (2d)</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver General</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Brooke Burnaby (2d)</t>
         </is>
@@ -1039,22 +1039,22 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>VMI Abbotsford/Langley (2d)</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Richmond</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>NSMI (4d)</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Comox</t>
+          <t>Mission</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>St.Paul's</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>WCMI Kerrisdale (2d)</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Royal Jubilee</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1082,35 +1082,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>UBC General</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Royal Jubilee</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>BCWH</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Peace Arch</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Vancouver General</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Delta</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>WCMI Hornby (2d)</t>
+          <t>Island ultrasound (5d)</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Burnaby (2d)</t>
         </is>
       </c>
     </row>
@@ -1135,35 +1135,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Royal Columbian</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Kamloops (RIH)</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Kelowna KGH</t>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Victoria</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Vancouver General/UBC</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Surrey</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>Vernon Radiology Associates (3d)</t>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Oceanside (Parksville) (5d)</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Vernon</t>
+          <t>NSMI Squamish (2d)</t>
         </is>
       </c>
     </row>
@@ -1188,35 +1188,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Burnaby</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>BCWH</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Richmond</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Richmond</t>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>St.Paul's</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>St.Paul's</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>MSJ</t>
+          <t>NSMI (4d)</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>UBC General</t>
+          <t>Island ultrasound (5d)</t>
         </is>
       </c>
     </row>
@@ -1241,35 +1241,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Kelowna KGH</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>BCWH</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Vancouver General/UBC</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Vancouver General/UBC</t>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Vernon</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Royal Columbian</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>Eagle Ridge</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver General</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>Brooke Burnaby (2d)</t>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Lindsay Diagnostics Kamloops (4d)</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Kamloops (RIH)</t>
+          <t>Greig Associates (2d)</t>
         </is>
       </c>
     </row>
@@ -1294,22 +1294,22 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>Royal Jubilee</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Chilliwack</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Victoria</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Ridge Meadows</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Nanaimo</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>UBC General</t>
         </is>
@@ -1317,12 +1317,12 @@
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Island ultrasound (5d)</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>Kamloops (RIH)</t>
+          <t>Chilliwack</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
         </is>
       </c>
     </row>
@@ -1349,33 +1349,33 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Penticton</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Abbotsford</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Surrey</t>
+          <t>BCWH</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Salmon Arm (SLDH)</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH)</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Vernon</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>WCMI Kerrisdale (2d)</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>Salmon Arm (SLDH)</t>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Victoria</t>
         </is>
       </c>
     </row>
@@ -1400,35 +1400,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>Richmond</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Lions Gate</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="F20" s="4" t="inlineStr">
         <is>
           <t>Burnaby</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
-        <is>
-          <t>Burnaby</t>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Campbell River</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver General</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>BCWH</t>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>NSMI Squamish (2d)</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Delta</t>
+          <t>Lindsay Diagnostics Kamloops (4d)</t>
         </is>
       </c>
     </row>
@@ -1455,33 +1455,33 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
+          <t>BCWH</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
           <t>Vernon</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Sechelt</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Royal Columbian</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Kamloops (RIH)</t>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Abbotsford</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>MSJ</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>Greig Associates (2d)</t>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>VMI Abbotsford/Langley (2d)</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>MSJ</t>
+          <t>Oceanside (Parksville) (5d)</t>
         </is>
       </c>
     </row>
@@ -1506,35 +1506,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Nanaimo</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>UBC General</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>MSJ</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Victoria</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>Campbell River</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Vancouver General</t>
+          <t>KMI Westside (3d)</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>NSMI (4d)</t>
+          <t>Chilliwack</t>
         </is>
       </c>
     </row>
@@ -1559,35 +1559,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Peace Arch</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Penticton</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Salmon Arm (SLDH)</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Kamloops (RIH)</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Penticton</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>Penticton</t>
-        </is>
-      </c>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>BCWH</t>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Richmond (4d)</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Mission</t>
+          <t>NSMI (4d)</t>
         </is>
       </c>
     </row>
@@ -1612,33 +1612,33 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
         <is>
           <t>Surrey</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Saanich</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>Campbell River</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Mission</t>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Royal Columbian</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Oceanside (Parksville) (5d)</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
+          <t>MSJ</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>BCWH</t>
         </is>
@@ -1665,35 +1665,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Vancouver General/UBC</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Nanaimo</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Eagle Ridge</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Kelowna KGH</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>Victoria</t>
         </is>
       </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Chilliwack</t>
+        </is>
+      </c>
       <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>Lindsay Diagnostics Kamloops (4d)</t>
-        </is>
-      </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>Comox</t>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Vernon Radiology Associates (3d)</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Richmond</t>
         </is>
       </c>
     </row>
@@ -1718,35 +1718,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Victoria</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Campbell River</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Peace Arch</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>Eagle Ridge</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Comox</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="6" t="inlineStr">
         <is>
           <t>BCWH</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>NSMI (4d)</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>Richmond</t>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>UBC General</t>
         </is>
       </c>
     </row>
@@ -1771,35 +1771,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>MSJ</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Penticton</t>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Kelowna KGH</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>BCWH</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>Royal Columbian</t>
+          <t>Ridge Meadows</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Ridge Meadows</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>Kelowna KGH</t>
-        </is>
-      </c>
-      <c r="K27" s="7" t="inlineStr">
-        <is>
-          <t>Kelowna KGH</t>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Greig Associates (2d)</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>VMI Abbotsford/Langley (2d)</t>
         </is>
       </c>
     </row>
@@ -1824,35 +1824,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Surrey</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>UBC General</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>Abbotsford</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Mission</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
         <is>
           <t>Royal Jubilee</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Vancouver General</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>Nanaimo</t>
-        </is>
-      </c>
-      <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>UBC General</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>Greig Associates (2d)</t>
         </is>
       </c>
     </row>
@@ -1877,35 +1877,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>MSJ</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Kamloops (RIH)</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Victoria</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>MSJ</t>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Vernon</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Lions Gate</t>
+          <t>BCWH</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>KMI R (2d)</t>
-        </is>
-      </c>
-      <c r="K29" s="3" t="inlineStr">
-        <is>
-          <t>Saanich</t>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>Kelowna KGH</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>Kelowna KGH</t>
         </is>
       </c>
     </row>
@@ -1930,35 +1930,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Campbell River</t>
-        </is>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>Eagle Ridge</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>UBC General</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>Abbotsford</t>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Comox</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Royal Jubilee</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>MSJ</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Royal Columbian</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>Medray (2d)</t>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Victoria</t>
+          <t>Vernon Radiology Associates (3d)</t>
         </is>
       </c>
     </row>
@@ -1983,35 +1983,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>UBC General</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Kelowna KGH</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>BCWH</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>Kamloops (RIH)</t>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Salmon Arm (SLDH)</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Vancouver General/UBC</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Penticton</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Penticton</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>Penticton</t>
+          <t>WCMI Hornby (2d)</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Chilliwack</t>
+          <t>KMI R (2d)</t>
         </is>
       </c>
     </row>
@@ -2036,35 +2036,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Chilliwack</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>Surrey</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Vancouver General/UBC</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>Abbotsford</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>BCWH</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>NSMI Squamish (2d)</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>Nanaimo</t>
+          <t>Vancouver General</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>Vernon</t>
         </is>
       </c>
     </row>
@@ -2089,35 +2089,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Lions Gate</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Ridge Meadows</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>Kamloops (RIH)</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>Vernon</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
-        <is>
-          <t>Surrey</t>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Kelowna KGH</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Kelowna KGH</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>VMI Abbotsford/Langley (2d)</t>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Medray (2d)</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Vancouver General</t>
+          <t>Brooke Richmond (4d)</t>
         </is>
       </c>
     </row>
@@ -2142,35 +2142,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>Comox</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>MSJ</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Royal Jubilee</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Abbotsford</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Lions Gate</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>Mission</t>
         </is>
       </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
-        </is>
-      </c>
       <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>Brooke Richmond (4d)</t>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Burnaby (2d)</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Vancouver General</t>
+          <t>WCMI Kerrisdale (2d)</t>
         </is>
       </c>
     </row>
@@ -2195,35 +2195,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>BCWH</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>Salmon Arm (SLDH)</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>Kelowna KGH</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>Vancouver General</t>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Penticton</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Eagle Ridge</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>Peace Arch</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>Peace Arch</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>Kamloops (RIH)</t>
+          <t>WCMI Kerrisdale (2d)</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Penticton</t>
+          <t>Medray (2d)</t>
         </is>
       </c>
     </row>
@@ -2248,35 +2248,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>Eagle Ridge</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Abbotsford</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Comox</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
         <is>
           <t>Burnaby</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>Delta</t>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Burnaby</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="4" t="inlineStr">
         <is>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
           <t>KMI Westside (3d)</t>
-        </is>
-      </c>
-      <c r="K36" s="3" t="inlineStr">
-        <is>
-          <t>Royal Jubilee</t>
         </is>
       </c>
     </row>
@@ -2301,35 +2301,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>Kamloops (RIH)</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>Vernon</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>Chilliwack</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>Peace Arch</t>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Nanaimo</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Langley</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Langley</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
-      <c r="J37" s="4" t="inlineStr">
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>KMI R (2d)</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
         <is>
           <t>WCMI Hornby (2d)</t>
-        </is>
-      </c>
-      <c r="K37" s="5" t="inlineStr">
-        <is>
-          <t>BCWH</t>
         </is>
       </c>
     </row>
@@ -2354,35 +2354,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>Royal Columbian</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="F38" s="4" t="inlineStr">
         <is>
           <t>Lions Gate</t>
         </is>
       </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>Eagle Ridge</t>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>UBC General</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>Squamish</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="3" t="inlineStr">
-        <is>
-          <t>Chilliwack</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr">
-        <is>
-          <t>Brooke Burnaby (2d)</t>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver General</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH)</t>
         </is>
       </c>
     </row>
@@ -2411,19 +2411,19 @@
       <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="J39" s="6" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Vancouver General/UBC</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
         <is>
           <t>Ridge Meadows</t>
         </is>
       </c>
-      <c r="K39" s="6" t="inlineStr">
-        <is>
-          <t>Peace Arch</t>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>Abbotsford</t>
         </is>
       </c>
     </row>
@@ -2452,19 +2452,19 @@
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>Langley</t>
-        </is>
-      </c>
-      <c r="J40" s="6" t="inlineStr">
-        <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="K40" s="6" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Burnaby</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>Vancouver General/UBC</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>Eagle Ridge</t>
         </is>
       </c>
     </row>
@@ -2493,19 +2493,19 @@
       <c r="F41" s="2" t="inlineStr"/>
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>Vancouver General/UBC</t>
-        </is>
-      </c>
-      <c r="J41" s="6" t="inlineStr">
-        <is>
-          <t>Abbotsford</t>
-        </is>
-      </c>
-      <c r="K41" s="6" t="inlineStr">
-        <is>
-          <t>Langley</t>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>St.Paul's</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>Eagle Ridge</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>Burnaby</t>
         </is>
       </c>
     </row>
@@ -2534,19 +2534,19 @@
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
-        </is>
-      </c>
-      <c r="J42" s="6" t="inlineStr">
-        <is>
-          <t>Langley</t>
-        </is>
-      </c>
-      <c r="K42" s="6" t="inlineStr">
-        <is>
-          <t>Royal Columbian</t>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>Abbotsford</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>Peace Arch</t>
         </is>
       </c>
     </row>
@@ -2575,19 +2575,19 @@
       <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
-        </is>
-      </c>
-      <c r="J43" s="6" t="inlineStr">
-        <is>
-          <t>Lions Gate</t>
-        </is>
-      </c>
-      <c r="K43" s="6" t="inlineStr">
-        <is>
-          <t>Surrey</t>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>Abbotsford</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>Langley</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>Royal Columbian</t>
         </is>
       </c>
     </row>
@@ -2616,19 +2616,19 @@
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>Peace Arch</t>
-        </is>
-      </c>
-      <c r="J44" s="6" t="inlineStr">
-        <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="K44" s="6" t="inlineStr">
-        <is>
-          <t>Vancouver General/UBC</t>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Royal Columbian</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>Burnaby</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>Langley</t>
         </is>
       </c>
     </row>
@@ -2657,19 +2657,19 @@
       <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="inlineStr"/>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="J45" s="6" t="inlineStr">
-        <is>
-          <t>Burnaby</t>
-        </is>
-      </c>
-      <c r="K45" s="6" t="inlineStr">
-        <is>
-          <t>Abbotsford</t>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>Ridge Meadows</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>Lions Gate</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>St.Paul's</t>
         </is>
       </c>
     </row>
@@ -2698,19 +2698,19 @@
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="6" t="inlineStr">
-        <is>
-          <t>Royal Columbian</t>
-        </is>
-      </c>
-      <c r="J46" s="6" t="inlineStr">
-        <is>
-          <t>Eagle Ridge</t>
-        </is>
-      </c>
-      <c r="K46" s="6" t="inlineStr">
-        <is>
-          <t>Burnaby</t>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Lions Gate</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>St.Paul's</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
         </is>
       </c>
     </row>
@@ -2739,19 +2739,19 @@
       <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr"/>
       <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="6" t="inlineStr">
-        <is>
-          <t>Burnaby</t>
-        </is>
-      </c>
-      <c r="J47" s="6" t="inlineStr">
-        <is>
-          <t>Royal Columbian</t>
-        </is>
-      </c>
-      <c r="K47" s="6" t="inlineStr">
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Eagle Ridge</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
         <is>
           <t>Surrey</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>Lions Gate</t>
         </is>
       </c>
     </row>
@@ -2780,19 +2780,19 @@
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="6" t="inlineStr">
-        <is>
-          <t>Eagle Ridge</t>
-        </is>
-      </c>
-      <c r="J48" s="6" t="inlineStr">
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>Peace Arch</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
         <is>
           <t>Vancouver General/UBC</t>
-        </is>
-      </c>
-      <c r="K48" s="6" t="inlineStr">
-        <is>
-          <t>Lions Gate</t>
         </is>
       </c>
     </row>
@@ -2821,19 +2821,19 @@
       <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr"/>
       <c r="H49" s="2" t="inlineStr"/>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>Lions Gate</t>
-        </is>
-      </c>
-      <c r="J49" s="6" t="inlineStr">
-        <is>
-          <t>Peace Arch</t>
-        </is>
-      </c>
-      <c r="K49" s="6" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>Langley</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>Royal Columbian</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
         </is>
       </c>
     </row>
@@ -2862,19 +2862,19 @@
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="6" t="inlineStr">
-        <is>
-          <t>Abbotsford</t>
-        </is>
-      </c>
-      <c r="J50" s="6" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
-        </is>
-      </c>
-      <c r="K50" s="6" t="inlineStr">
-        <is>
-          <t>Eagle Ridge</t>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Peace Arch</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>Ridge Meadows</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
new version applying fixes from feedback
</commit_message>
<xml_diff>
--- a/Generated_Schedule.xlsx
+++ b/Generated_Schedule.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,22 +544,22 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>NSMI (4d)</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Surrey</t>
+          <t>Greig Associates* (2d)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>WCMI* (2d)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>WCMI Hornby (2d)</t>
+          <t>NSMI* (4d)</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Brooke Richmond (4d)</t>
+          <t>Brooke Burnaby* (2d)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -587,24 +587,24 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Chilliwack</t>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>VMI Abbotsford/Langley* (2d)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Medray (2d)</t>
+          <t>NSMI (4d)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Brooke Richmond (4d)</t>
+          <t>Brooke Richmond* (4d)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>VMI Abbotsford/Langley (2d)</t>
+          <t>Medray* (2d)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -634,22 +634,22 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Brooke Burnaby (2d)</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Richmond</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver General</t>
+          <t>NSMI* (4d)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Burnaby* (2d)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Vernon Radiology Associates (3d)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Greig Associates (2d)</t>
+          <t>NSMI Squamish* (2d)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -677,24 +677,24 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Mission</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Burnaby* (2d)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Greig Associates (2d)</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Chilliwack</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Burnaby</t>
+          <t>Greig Associates* (2d)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>NSMI Squamish (2d)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Richmond (4d)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -722,24 +722,24 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Cranbrook (EKRH)</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver General</t>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>WCMI* (2d)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Richmond* (4d)</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>VMI Abbotsford/Langley (2d)</t>
+          <t>Brooke Burnaby (2d)</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>NSMI (4d)</t>
+          <t>Vernon Radiology Associates (3d)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -769,22 +769,22 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Brooke Richmond (4d)</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Burnaby</t>
+          <t>NSMI Squamish (2d)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Medray* (2d)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Brooke Burnaby (2d)</t>
+          <t>VMI Abbotsford/Langley* (2d)</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Medray (2d)</t>
+          <t>Greig Associates* (2d)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -812,24 +812,24 @@
           <t>General</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Delta</t>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Medray* (2d)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Brooke Richmond (4d)</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver General</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>UBC General</t>
+          <t>KMI (2d)</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Greig Associates* (2d)</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>WCMI* (2d)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -859,22 +859,22 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Langley</t>
+          <t>Mission</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Brooke Burnaby (2d)</t>
+          <t>VMI Abbotsford/Langley* (2d)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Greig Associates (2d)</t>
+          <t>Medray* (2d)</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>WCMI Kerrisdale (2d)</t>
+          <t>NSMI (4d)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -904,22 +904,22 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Greig Associates (2d)</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver General</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Richmond</t>
+          <t>Brooke Richmond* (4d)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>NSMI Squamish (2d)</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>WCMI* (2d)</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>WCMI Hornby (2d)</t>
+          <t>VMI Abbotsford/Langley (2d)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -949,33 +949,33 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
+          <t>Royal Columbian*</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Peace Arch</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
           <t>Surrey</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Sechelt</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>Mission</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Eagle Ridge</t>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>BCWH*</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>Medray (2d)</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>Comox</t>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Delta</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Lindsay Diagnostics Kamloops (4d)</t>
         </is>
       </c>
     </row>
@@ -1000,35 +1000,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Vernon</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Peace Arch</t>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Salmon Arm (SLDH)*</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Lindsay Diagnostics Kamloops* (4d)</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>UBC General</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Delta</t>
+          <t>Richmond</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>WCMI Kerrisdale (2d)</t>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Vernon*</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>Victoria</t>
+          <t>Comox</t>
         </is>
       </c>
     </row>
@@ -1053,35 +1053,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Richmond</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>Burnaby</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Chilliwack</t>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Langley*</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Langley*</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>BCWH*</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Peace Arch</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>Vancouver General</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>VMI Abbotsford/Langley* (2d)</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>Campbell River</t>
         </is>
       </c>
     </row>
@@ -1108,33 +1108,33 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Kamloops (RIH)</t>
+          <t>Kamloops (RIH)*</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Kamloops (RIH)</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Squamish</t>
+          <t>Penticton*</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Nanaimo</t>
+          <t>Vernon*</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Greig Associates (2d)</t>
+          <t>Brooke Richmond (4d)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>Vernon</t>
+          <t>Victoria</t>
         </is>
       </c>
     </row>
@@ -1159,35 +1159,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>UBC General</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Vancouver General/UBC</t>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Abbotsford</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Ridge Meadows</t>
+          <t>Lions Gate</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Comox</t>
+          <t>Surrey</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Brooke Richmond (4d)</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
+          <t>Island ultrasound* (5d)</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Greig Associates (2d)</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>MSJ</t>
+          <t>Penticton*</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Penticton</t>
+          <t>Abbotsford</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1229,18 +1229,18 @@
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Vancouver General</t>
+          <t>Eagle Ridge</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Oceanside (Parksville) (5d)</t>
+          <t>Lindsay Diagnostics Kamloops (4d)</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Brooke Richmond (4d)</t>
+          <t>KMI* (2d)</t>
         </is>
       </c>
     </row>
@@ -1267,33 +1267,33 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>BCWH</t>
+          <t>BCWH*</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Surrey</t>
+          <t>Vancouver General/UBC</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Langley</t>
+          <t>Kamloops (RIH)</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Vancouver General</t>
+          <t>Vancouver General*</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>MSJ</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Chilliwack</t>
+          <t>Mission</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>NSMI Squamish (2d)</t>
         </is>
       </c>
     </row>
@@ -1318,35 +1318,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Kelowna KGH*</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Kamloops (RIH)</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>Vernon</t>
+          <t>Lions Gate</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>MSJ</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Abbotsford</t>
+          <t>MSJ</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>KMI R (2d)</t>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH)*</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Lindsay Diagnostics Kamloops (4d)</t>
+          <t>NSMI (4d)</t>
         </is>
       </c>
     </row>
@@ -1371,35 +1371,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Sechelt</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>Lions Gate</t>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Eagle Ridge</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>UBC General</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Surrey</t>
+          <t>Ridge Meadows</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Royal Jubilee</t>
+          <t>Nanaimo*</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>NSMI Squamish (2d)</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Vernon Radiology Associates (3d)</t>
+          <t>Brooke Richmond (4d)</t>
         </is>
       </c>
     </row>
@@ -1424,35 +1424,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Vernon Radiology Associates* (3d)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Salmon Arm (SLDH)</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>Penticton</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>MSJ</t>
+          <t>Mission</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Chilliwack</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Abbotsford</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>Mission</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>Medray (2d)</t>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>NSMI (4d)</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Vernon*</t>
         </is>
       </c>
     </row>
@@ -1477,35 +1477,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Abbotsford</t>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>BCWH*</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Langley</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>Peace Arch</t>
+          <t>Ridge Meadows</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>Burnaby</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Vancouver General*</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>Vernon Radiology Associates (3d)</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>Greig Associates (2d)</t>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>MSJ</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Richmond</t>
         </is>
       </c>
     </row>
@@ -1530,35 +1530,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Kelowna KGH</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Richmond</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH)*</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Kelowna KGH*</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Royal Columbian</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>UBC General</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>NSMI (4d)</t>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Brooke Burnaby (2d)</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Eagle Ridge</t>
+          <t>Ridge Meadows</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1595,23 +1595,23 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Abbotsford</t>
+          <t>Surrey</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Victoria</t>
+          <t>Comox*</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>NSMI Squamish (2d)</t>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>KMI R (2d)</t>
+          <t>Oceanside (Parksville)* (5d)</t>
         </is>
       </c>
     </row>
@@ -1636,35 +1636,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>KMI* (2d)</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Peace Arch</t>
+          <t>Penticton*</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>Kamloops (RIH)</t>
+          <t>Ridge Meadows</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Vernon</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>WCMI Kerrisdale (2d)</t>
+          <t>Chilliwack</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
         </is>
       </c>
     </row>
@@ -1689,35 +1689,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>Burnaby</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>St.Paul's*</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>St.Paul's*</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Surrey</t>
+          <t>Royal Columbian*</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>Surrey</t>
+          <t>Chilliwack</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>Chilliwack</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
           <t>UBC General</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Island ultrasound (5d)</t>
         </is>
       </c>
     </row>
@@ -1742,35 +1742,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Kamloops (RIH)</t>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Lindsay Diagnostics Kamloops* (4d)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Vernon</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
+          <t>Royal Columbian</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Vancouver General/UBC</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Surrey</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>KMI Westside (3d)</t>
+          <t>Oceanside (Parksville) (5d)</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>NSMI Squamish (2d)</t>
+          <t>Medray (2d)</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Squamish</t>
+          <t>Lions Gate</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -1807,23 +1807,23 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Lions Gate</t>
+          <t>Abbotsford</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>Campbell River</t>
+          <t>Royal Jubilee*</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>WCMI (2d)</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>WCMI Hornby (2d)</t>
+          <t>Brooke Burnaby (2d)</t>
         </is>
       </c>
     </row>
@@ -1850,33 +1850,33 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Salmon Arm (SLDH)</t>
+          <t>Surrey</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Kelowna KGH</t>
+          <t>Kamloops (RIH)*</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Vancouver General/UBC</t>
+          <t>Vernon*</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Vancouver General/UBC</t>
+          <t>Delta</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>NSMI (4d)</t>
-        </is>
-      </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>KMI Westside (3d)</t>
+          <t>KMI* (2d)</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
         </is>
       </c>
     </row>
@@ -1901,35 +1901,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>UBC General*</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>Surrey</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Mission</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>MSJ</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Langley</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>BCWH*</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="4" t="inlineStr">
         <is>
           <t>Richmond</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>Brooke Burnaby (2d)</t>
-        </is>
-      </c>
-      <c r="K29" s="5" t="inlineStr">
-        <is>
-          <t>Campbell River</t>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Vernon Radiology Associates (3d)</t>
         </is>
       </c>
     </row>
@@ -1956,33 +1956,33 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Vancouver General/UBC</t>
+          <t>Vernon*</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
+          <t>MSJ</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
           <t>UBC General</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>Kamloops (RIH)</t>
-        </is>
-      </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Vernon</t>
+          <t>Kamloops (RIH)*</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>Lindsay Diagnostics Kamloops (4d)</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>Island ultrasound (5d)</t>
+          <t>Greig Associates (2d)</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>Surrey</t>
         </is>
       </c>
     </row>
@@ -2009,33 +2009,33 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Lions Gate</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Abbotsford</t>
+          <t>Surrey</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>BCWH</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Royal Columbian</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>BCWH</t>
+          <t>Peace Arch</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Victoria*</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>Victoria</t>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Vernon Radiology Associates (3d)</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>VMI Abbotsford/Langley (2d)</t>
+          <t>WCMI (2d)</t>
         </is>
       </c>
     </row>
@@ -2060,35 +2060,35 @@
           <t>Dual</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Penticton</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Royal Columbian</t>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Vancouver General/UBC</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Vernon*</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Kamloops (RIH)</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Surrey</t>
+          <t>Mission</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>UBC General</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>Island ultrasound (5d)</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>Brooke Burnaby (2d)</t>
+          <t>Medray (2d)</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH)*</t>
         </is>
       </c>
     </row>
@@ -2115,103 +2115,91 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Peace Arch</t>
+          <t>Kamloops (RIH)*</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Delta</t>
+          <t>Kelowna KGH*</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Kelowna KGH</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
+          <t>St.Paul's</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Lions Gate</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="6" t="inlineStr">
         <is>
           <t>BCWH</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>WCMI Hornby (2d)</t>
-        </is>
-      </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Oceanside (Parksville) (5d)</t>
+          <t>VMI Abbotsford/Langley (2d)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>638205</t>
+          <t>STU1003</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Kathie</t>
+          <t>Brown</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bron </t>
+          <t>Sophia</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Dual</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Royal Columbian</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>MSJ</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>Delta</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>Lions Gate</t>
-        </is>
-      </c>
-      <c r="I34" s="2" t="inlineStr"/>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>VMI Abbotsford/Langley (2d)</t>
+          <t>Cardiac</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>St.Paul's*</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>Abbotsford*</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>Royal Jubilee</t>
+          <t>Burnaby</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>STU1003</t>
+          <t>STU1007</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Brown</t>
+          <t>Taylor</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Sophia</t>
+          <t>Ava</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2225,34 +2213,34 @@
       <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>Royal Columbian</t>
+          <t>Eagle Ridge</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>Peace Arch</t>
+          <t>Vancouver General/UBC*</t>
         </is>
       </c>
       <c r="K35" s="5" t="inlineStr">
         <is>
-          <t>Vancouver General/UBC</t>
+          <t>Lions Gate*</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>STU1007</t>
+          <t>STU1011</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Taylor</t>
+          <t>White</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Ava</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2266,34 +2254,34 @@
       <c r="H36" s="2" t="inlineStr"/>
       <c r="I36" s="5" t="inlineStr">
         <is>
+          <t>Abbotsford*</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>Burnaby*</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
           <t>Eagle Ridge</t>
-        </is>
-      </c>
-      <c r="J36" s="5" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
-        </is>
-      </c>
-      <c r="K36" s="5" t="inlineStr">
-        <is>
-          <t>Abbotsford</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>STU1011</t>
+          <t>STU1015</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>White</t>
+          <t>Garcia</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>Mia</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2307,34 +2295,34 @@
       <c r="H37" s="2" t="inlineStr"/>
       <c r="I37" s="5" t="inlineStr">
         <is>
+          <t>Burnaby*</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>Surrey*</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
           <t>Peace Arch</t>
-        </is>
-      </c>
-      <c r="J37" s="5" t="inlineStr">
-        <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="K37" s="5" t="inlineStr">
-        <is>
-          <t>Lions Gate</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>STU1015</t>
+          <t>STU1019</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Garcia</t>
+          <t>Rodriguez</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Mia</t>
+          <t>Abigail</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2348,34 +2336,34 @@
       <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Burnaby</t>
+          <t>Ridge Meadows</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Langley</t>
+          <t>St.Paul's*</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
         <is>
-          <t>Royal Columbian</t>
+          <t>Vancouver General/UBC*</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>STU1019</t>
+          <t>STU1023</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Rodriguez</t>
+          <t>Hall</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Abigail</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2389,34 +2377,34 @@
       <c r="H39" s="2" t="inlineStr"/>
       <c r="I39" s="5" t="inlineStr">
         <is>
+          <t>Langley*</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
           <t>Ridge Meadows</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>Vancouver General/UBC</t>
-        </is>
-      </c>
       <c r="K39" s="5" t="inlineStr">
         <is>
-          <t>Surrey</t>
+          <t>St.Paul's*</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>STU1023</t>
+          <t>STU1027</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Hall</t>
+          <t>Wright</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Mila</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2430,34 +2418,34 @@
       <c r="H40" s="2" t="inlineStr"/>
       <c r="I40" s="5" t="inlineStr">
         <is>
+          <t>Surrey*</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>Lions Gate*</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
           <t>Langley</t>
-        </is>
-      </c>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>Surrey</t>
-        </is>
-      </c>
-      <c r="K40" s="5" t="inlineStr">
-        <is>
-          <t>Kamloops (RIH)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>STU1027</t>
+          <t>STU1031</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Wright</t>
+          <t>Adams</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Mila</t>
+          <t>Chloe</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2471,34 +2459,34 @@
       <c r="H41" s="2" t="inlineStr"/>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>Vancouver General/UBC</t>
+          <t>Royal Columbian*</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>Abbotsford</t>
+          <t>Surrey*</t>
         </is>
       </c>
       <c r="K41" s="5" t="inlineStr">
         <is>
-          <t>Ridge Meadows</t>
+          <t>Nanaimo</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>STU1031</t>
+          <t>STU1035</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Adams</t>
+          <t>Perez</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Chloe</t>
+          <t>Zoey</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2512,34 +2500,34 @@
       <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Surrey</t>
+          <t>Lions Gate*</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>Eagle Ridge</t>
+          <t>Peace Arch</t>
         </is>
       </c>
       <c r="K42" s="5" t="inlineStr">
         <is>
-          <t>Burnaby</t>
+          <t>Royal Columbian*</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>STU1035</t>
+          <t>STU1039</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Perez</t>
+          <t>Campbell</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Zoey</t>
+          <t>Victoria</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2553,34 +2541,34 @@
       <c r="H43" s="2" t="inlineStr"/>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Abbotsford</t>
+          <t>Peace Arch*</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>Royal Columbian</t>
+          <t>Langley*</t>
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr">
         <is>
-          <t>Surrey</t>
+          <t>Ridge Meadows</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>STU1039</t>
+          <t>STU1043</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Campbell</t>
+          <t>Collins</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Victoria</t>
+          <t>Hannah</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2594,34 +2582,34 @@
       <c r="H44" s="2" t="inlineStr"/>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Surrey</t>
+          <t>Vancouver General/UBC*</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>Burnaby</t>
+          <t>Royal Columbian*</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
         <is>
-          <t>Eagle Ridge</t>
+          <t>Abbotsford</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>STU1043</t>
+          <t>STU1047</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Collins</t>
+          <t>Rogers</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Hannah</t>
+          <t>Layla</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2635,58 +2623,822 @@
       <c r="H45" s="2" t="inlineStr"/>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>St.Paul's</t>
+          <t>Surrey*</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>Lions Gate</t>
+          <t>Eagle Ridge*</t>
         </is>
       </c>
       <c r="K45" s="5" t="inlineStr">
         <is>
-          <t>Peace Arch</t>
+          <t>Royal Jubilee</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>STU1047</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Rogers</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>Layla</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>Cardiac</t>
-        </is>
-      </c>
+      <c r="A46" s="2" t="inlineStr"/>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="5" t="inlineStr">
-        <is>
-          <t>Lions Gate</t>
-        </is>
-      </c>
-      <c r="J46" s="5" t="inlineStr">
-        <is>
-          <t>Ridge Meadows</t>
-        </is>
-      </c>
-      <c r="K46" s="5" t="inlineStr">
-        <is>
-          <t>St.Paul's</t>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>UNUSED SITES</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Burnaby (1)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Burnaby (1)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Cranbrook (EKRH) (1)</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Burnaby (1)</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>BCWH (2)</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Campbell River (1)</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Chilliwack (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Burnaby (1)</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Burnaby (1)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Delta (1)</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Burnaby (1)</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Campbell River (1)</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Campbell River (1)</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Cranbrook (EKRH) (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Chilliwack (1)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Cranbrook (EKRH) (1)</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH) (1)</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Campbell River (1)</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Campbell River (1)</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Comox (1)</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Delta (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Cranbrook (EKRH) (1)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Delta (1)</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Salmon Arm (SLDH) (1)</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Campbell River (1)</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Chilliwack (1)</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Comox (1)</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Duncan (CDH) (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Delta (1)</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Richmond (1)</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Sechelt (1)</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Cranbrook (EKRH) (1)</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Comox (1)</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Cranbrook (EKRH) (1)</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH) (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>MSJ (1)</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Salmon Arm (SLDH) (1)</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Squamish (1)</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Duncan (CDH) (1)</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Comox (1)</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Duncan (CDH) (1)</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Kelowna KGH (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Peace Arch (1)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Sechelt (1)</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Vancouver General (2)</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH) (1)</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Cranbrook (EKRH) (1)</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH) (1)</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Kelowna KGH (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Peace Arch (1)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Squamish (1)</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>KMI (Open)</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Kelowna KGH (1)</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Delta (1)</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Kelowna KGH (1)</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Mission (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Sechelt (1)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Vancouver General (2)</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Lindsay Diagnostics Kamloops (Open)</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Kelowna KGH (1)</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Duncan (CDH) (1)</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Kelowna KGH (1)</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>MSJ (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Squamish (1)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Vernon Radiology Associates (Open)</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Langley (1)</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH) (2)</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Nanaimo (1)</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Penticton (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Vancouver General (2)</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Langley (1)</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Kamloops (RIH) (1)</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Nanaimo (1)</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Penticton (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Mission (1)</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Kelowna KGH (1)</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Penticton (1)</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Saanich (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Penticton (1)</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Kelowna KGH (1)</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Penticton (1)</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Salmon Arm (SLDH) (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Penticton (1)</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Mission (1)</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Royal Jubilee (1)</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Sechelt (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Saanich (1)</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>MSJ (1)</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Royal Jubilee (1)</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Squamish (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Salmon Arm (SLDH) (1)</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Nanaimo (1)</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Saanich (1)</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>UBC General (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Sechelt (1)</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Nanaimo (1)</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Salmon Arm (SLDH) (1)</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Vancouver General (2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Squamish (1)</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Penticton (1)</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>Sechelt (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>St.Paul's (1)</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Penticton (1)</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Squamish (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>St.Paul's (1)</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Richmond (1)</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>Vancouver General (2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Vancouver General/UBC (1)</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Royal Jubilee (1)</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Victoria (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Island ultrasound (Open)</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Royal Jubilee (1)</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Victoria (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>KMI (Open)</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Saanich (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Lindsay Diagnostics Kamloops (Open)</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Salmon Arm (SLDH) (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Oceanside (Parksville) (Open)</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Sechelt (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Squamish (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>UBC General (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Vancouver General (2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Vernon (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Vernon (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Victoria (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Victoria (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Brooke Burnaby (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Brooke Richmond (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Greig Associates (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Island ultrasound (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>KMI (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Lindsay Diagnostics Kamloops (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Medray (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>NSMI (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>NSMI Squamish (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Oceanside (Parksville) (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Vernon Radiology Associates (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>VMI Abbotsford/Langley (Open)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>WCMI (Open)</t>
         </is>
       </c>
     </row>

</xml_diff>